<commit_message>
fixed srs 1.1 and requirements defects
</commit_message>
<xml_diff>
--- a/docs/sprint2/requirements-defects.xlsx
+++ b/docs/sprint2/requirements-defects.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\turez\Desktop\sprint2\docs\sprint2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivasa\fb44_autorate\docs\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4664195-7A4E-4A1C-9F72-1B78F9D81D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Реєстр" sheetId="1" r:id="rId1"/>
@@ -21,12 +22,23 @@
     <sheet name="СМ_аудит" sheetId="7" r:id="rId7"/>
     <sheet name="КТ_аудит" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="329">
   <si>
     <t>№</t>
   </si>
@@ -46,9 +58,6 @@
     <t>Пропозиція виправлення</t>
   </si>
   <si>
-    <t>Хто знайшов (відповідальний)</t>
-  </si>
-  <si>
     <t>Статус</t>
   </si>
   <si>
@@ -67,15 +76,9 @@
     <t>«Popular Make/Popular Model» — немає однозначного правила визначення популярності та розв’язання нічиєї.</t>
   </si>
   <si>
-    <t>Обрати за кількістю голосів; за однакових значень сортувати за назвою.</t>
-  </si>
-  <si>
     <t>Асташов Іван</t>
   </si>
   <si>
-    <t>прийнято</t>
-  </si>
-  <si>
     <t>RD-01</t>
   </si>
   <si>
@@ -88,9 +91,6 @@
     <t>«достатньо складним» не дає єдиного трактування правила пароля.</t>
   </si>
   <si>
-    <t>Встановити довжину 8–64, щонайменше 1 латинська літера і 1 цифра.</t>
-  </si>
-  <si>
     <t>Кінаш Єгор</t>
   </si>
   <si>
@@ -103,9 +103,6 @@
     <t>«належним чином» не вказує, за яких саме умов кнопка Register активна.</t>
   </si>
   <si>
-    <t>Увімкнення лише після заповнення полів, збігу паролів та перевірки F-30.</t>
-  </si>
-  <si>
     <t>Рушай Євген</t>
   </si>
   <si>
@@ -121,9 +118,6 @@
     <t>«окреме слово» у стоп-списку не визначає межі слова і поведінку щодо «spam!» / «spammer».</t>
   </si>
   <si>
-    <t>Визначити слова послідовністю літер Unicode і розділювачі та приклади збігу.</t>
-  </si>
-  <si>
     <t>Дарина Поломарьова</t>
   </si>
   <si>
@@ -142,9 +136,6 @@
     <t>Не описано, що відбувається за неправильного логіна або пароля (сама GUI-30 визначає тільки розміщення повідомлення).</t>
   </si>
   <si>
-    <t>Не входити, лишити поточну сторінку, показати «Invalid login or password».</t>
-  </si>
-  <si>
     <t>RD-05</t>
   </si>
   <si>
@@ -154,9 +145,6 @@
     <t>Не визначено стан таблиці/пагінації, якщо моделей 0.</t>
   </si>
   <si>
-    <t>Показати «No models found», приховати елементи пагінації.</t>
-  </si>
-  <si>
     <t>RD-06</t>
   </si>
   <si>
@@ -166,9 +154,6 @@
     <t>Для сортування за rating не визначено порядок моделей з однаковим рейтингом.</t>
   </si>
   <si>
-    <t>Додати вторинне сортування за повною назвою без урахування регістру.</t>
-  </si>
-  <si>
     <t>RD-07</t>
   </si>
   <si>
@@ -181,9 +166,6 @@
     <t>Посилання на «АР-СТД-07», який не надано, робить неможливою перевірку довідки.</t>
   </si>
   <si>
-    <t>Замінити відсутній документ переліком 5 розділів і вимог до змісту довідки.</t>
-  </si>
-  <si>
     <t>RD-08</t>
   </si>
   <si>
@@ -199,9 +181,6 @@
     <t>Ранг визначається кількістю голосів, а F-130 — рейтингом за BL-10.</t>
   </si>
   <si>
-    <t>Ранг у F-60 визначити за зваженим рейтингом, tie-break як BL-20.</t>
-  </si>
-  <si>
     <t>RD-09</t>
   </si>
   <si>
@@ -211,9 +190,6 @@
     <t>BL-50 дозволяє порожній коментар/null, F-90 забороняє голос без коментаря.</t>
   </si>
   <si>
-    <t>BL-50 відхиляє null, порожній і пробільний коментар.</t>
-  </si>
-  <si>
     <t>RD-10</t>
   </si>
   <si>
@@ -223,9 +199,6 @@
     <t>Мінімальний поріг у F-130 — 5 голосів, а у BL-20 — 3 голоси.</t>
   </si>
   <si>
-    <t>У F-130 прийняти поріг 3 голоси і погодити F-60 з BL-20.</t>
-  </si>
-  <si>
     <t>RD-11</t>
   </si>
   <si>
@@ -235,9 +208,6 @@
     <t>GUI-60 задає 10 рядків на сторінці, F-140 — 5 рядків.</t>
   </si>
   <si>
-    <t>GUI-60: 5 рядків; узгодити з F-140.</t>
-  </si>
-  <si>
     <t>RD-12</t>
   </si>
   <si>
@@ -250,9 +220,6 @@
     <t>У межах однієї вимоги сеанс «безстроковий» і одночасно закінчується через 30 хвилин.</t>
   </si>
   <si>
-    <t>30 хвилин бездіяльності або Logout; активність скидає таймер.</t>
-  </si>
-  <si>
     <t>RD-13</t>
   </si>
   <si>
@@ -268,9 +235,6 @@
     <t>Дві різні вимоги з однаковим ідентифікатором GUI-40.</t>
   </si>
   <si>
-    <t>Зберегти першу GUI-40, другу позначити новим GUI-45 між GUI-40 і GUI-50.</t>
-  </si>
-  <si>
     <t>RD-14</t>
   </si>
   <si>
@@ -280,9 +244,6 @@
     <t>Вимога «Паролі користувачів зберігаються лише у вигляді хешу» стоїть без ID.</t>
   </si>
   <si>
-    <t>Призначити новий ID S-15, без зміни наявних ID.</t>
-  </si>
-  <si>
     <t>RD-15</t>
   </si>
   <si>
@@ -295,9 +256,6 @@
     <t>F-120 повторює функціональність F-70 і частину F-10 про Overall Rating.</t>
   </si>
   <si>
-    <t>Вилучити дубль F-120, зберегти F-70 і зафіксувати вилучення в журналі.</t>
-  </si>
-  <si>
     <t>RD-16</t>
   </si>
   <si>
@@ -307,9 +265,6 @@
     <t>Посилання на BL-35, якого немає у SRS (наявний BL-30).</t>
   </si>
   <si>
-    <t>Замінити посилання в F-100 на BL-30.</t>
-  </si>
-  <si>
     <t>RD-17</t>
   </si>
   <si>
@@ -322,9 +277,6 @@
     <t>Перевірка адреси, телефону й віку за державними реєстрами вимагає недоступних інтеграцій.</t>
   </si>
   <si>
-    <t>Перевіряти локально формат телефону, діапазон віку і довжину адреси.</t>
-  </si>
-  <si>
     <t>RD-18</t>
   </si>
   <si>
@@ -334,18 +286,12 @@
     <t>Розпізнавання будь-яких друкарських помилок, транслітерації й наміру будь-якою мовою неможливо гарантувати.</t>
   </si>
   <si>
-    <t>Залишити точний пошук за префіксом без регістру, явно виключити семантичні обіцянки.</t>
-  </si>
-  <si>
     <t>RD-19</t>
   </si>
   <si>
     <t>«працювати без помилок за будь-яких вхідних даних» не враховує помилкові аргументи.</t>
   </si>
   <si>
-    <t>Уточнити перевірки та передбачені винятки для некоректних даних.</t>
-  </si>
-  <si>
     <t>RD-20</t>
   </si>
   <si>
@@ -355,9 +301,6 @@
     <t>50 мс навіть через 2G і незалежно від розміру каталогу технічно не гарантовані.</t>
   </si>
   <si>
-    <t>Визначити контрольоване середовище, ≤1 000 моделей, p95 ≤3 с.</t>
-  </si>
-  <si>
     <t>RD-21</t>
   </si>
   <si>
@@ -373,9 +316,6 @@
     <t>«зручно ... не викликати труднощів» не має спостережуваного критерію проходження.</t>
   </si>
   <si>
-    <t>Перевірити 5 користувачів: ≥4 завершують редагування ≤3 хв.</t>
-  </si>
-  <si>
     <t>RD-22</t>
   </si>
   <si>
@@ -385,9 +325,6 @@
     <t>«працювати швидко» — відсутні одиниці вимірювання й умови.</t>
   </si>
   <si>
-    <t>p95 відкриття моделі ≤2,5 с, підтвердження голосу ≤2 с, по 30 замірів.</t>
-  </si>
-  <si>
     <t>RD-23</t>
   </si>
   <si>
@@ -397,9 +334,6 @@
     <t>«інтуїтивно ... для будь-якого» неможливо перевірити з відтворюваним результатом.</t>
   </si>
   <si>
-    <t>≥4 із 5 новачків знаходять модель і голосування ≤3 хв.</t>
-  </si>
-  <si>
     <t>RD-24</t>
   </si>
   <si>
@@ -409,9 +343,6 @@
     <t>«унеможливити будь-які спроби доступу» не дозволяє скінченного набору перевірок.</t>
   </si>
   <si>
-    <t>Конкретні відмови для гостя й правило 5 помилок /15 хв → 15 хв блокування.</t>
-  </si>
-  <si>
     <t>RD-25</t>
   </si>
   <si>
@@ -481,105 +412,57 @@
     <t>F-130 / BL-20</t>
   </si>
   <si>
-    <t>3 проти 5 голосів</t>
-  </si>
-  <si>
     <t>BL-20 задає поріг 3, F-130 — 5</t>
   </si>
   <si>
-    <t>Робоче значення 3</t>
-  </si>
-  <si>
-    <t>Підтвердити із замовником</t>
-  </si>
-  <si>
     <t>Q-02</t>
   </si>
   <si>
     <t>F-60 / F-130</t>
   </si>
   <si>
-    <t>ранг за голосами чи rating</t>
-  </si>
-  <si>
     <t>Замовлена функція рейтингу тижня використовує зважені оцінки</t>
   </si>
   <si>
-    <t>Ранг за рейтингом, popular за голосами</t>
-  </si>
-  <si>
     <t>Q-03</t>
   </si>
   <si>
-    <t>складність пароля</t>
-  </si>
-  <si>
     <t>«достатньо складним» не має чисел</t>
   </si>
   <si>
-    <t>8–64 + латинська літера й цифра</t>
-  </si>
-  <si>
     <t>Q-04</t>
   </si>
   <si>
     <t>S-10 / S-20</t>
   </si>
   <si>
-    <t>підбір пароля і сеанс</t>
-  </si>
-  <si>
     <t>Не задано конкретної кількості спроб у S-10</t>
   </si>
   <si>
-    <t>5 помилок /15 хв, блок 15 хв; таймаут 30 хв</t>
-  </si>
-  <si>
     <t>Q-05</t>
   </si>
   <si>
     <t>P-10 / P-20</t>
   </si>
   <si>
-    <t>пороги часу і середовище</t>
-  </si>
-  <si>
     <t>50 мс навіть на 2G недосяжне</t>
   </si>
   <si>
-    <t>p95 ≤3 с для рейтингу; P-20 за уточненням</t>
-  </si>
-  <si>
     <t>Q-06</t>
   </si>
   <si>
-    <t>повторення F-70</t>
-  </si>
-  <si>
     <t>Дві вимоги описують один список рейтингів</t>
   </si>
   <si>
-    <t>Вилучити F-120, зберігати пропуск нумерації</t>
-  </si>
-  <si>
-    <t>Запропоновано</t>
-  </si>
-  <si>
     <t>Q-07</t>
   </si>
   <si>
     <t>BL-50 / F-90</t>
   </si>
   <si>
-    <t>порожній коментар</t>
-  </si>
-  <si>
     <t>UI не приймає, а модуль приймає</t>
   </si>
   <si>
-    <t>Заборонити null/порожній/пробільний коментар</t>
-  </si>
-  <si>
     <t>Кількість дефектів</t>
   </si>
   <si>
@@ -607,187 +490,547 @@
     <t>Розглянуто типів</t>
   </si>
   <si>
-    <t>Кандидат № — Асташов Іван</t>
-  </si>
-  <si>
-    <t>Що перевірити</t>
-  </si>
-  <si>
-    <t>Статус незалежного аудиту</t>
-  </si>
-  <si>
-    <t>Власний висновок</t>
-  </si>
-  <si>
-    <t>Дата/підпис</t>
-  </si>
-  <si>
-    <t>перевірити незалежно</t>
-  </si>
-  <si>
-    <t>Кандидат № — Кінаш Єгор</t>
-  </si>
-  <si>
-    <t>Кандидат № — Рушай Євген</t>
-  </si>
-  <si>
-    <t>Кандидат № — Дарина Поломарьова</t>
-  </si>
-  <si>
-    <t>Зараз не зрозуміло, як саме обираються Popular Make і Popular Model при однаковій кількості голосів. Пропоную визначати популярність за голосами, а при нічиїй сортувати назви за алфавітом. Це дає одне очікуване значення для обох блоків.</t>
-  </si>
-  <si>
-    <t>Фраза «достатньо складний пароль» допускає різні перевірки. Потрібно прямо записати умови: 8–64 символи, щонайменше одна латинська літера та одна цифра. Тоді можна скласти позитивні й негативні тест-кейси.</t>
-  </si>
-  <si>
-    <t>У F-40 описаний лише успішний вхід. Для помилки треба додати відмову в авторизації, збереження поточної сторінки та повідомлення «Invalid login or password». Це необхідно для перевірки негативного сценарію.</t>
-  </si>
-  <si>
-    <t>Не описано, як виглядає рейтинг, коли немає жодної моделі. Пропоную показувати «No models found» і не відображати кнопки пагінації, щоб не було порожніх сторінок. Так можна перевірити порожню вибірку.</t>
-  </si>
-  <si>
-    <t>D-10 посилається на документ АР-СТД-07, якого немає серед матеріалів. Краще перелічити обов’язкові розділи довідки в самій SRS, щоб вимогу можна було перевірити. Інакше вимогу до довідки неможливо оцінити.</t>
-  </si>
-  <si>
-    <t>У F-60 ранг залежить від кількості голосів, але F-130 використовує зважений рейтинг. Потрібно встановити єдине правило ранжування за рейтингом і узгодити його з BL-20. Однакове правило потрібне для тестів рейтингу.</t>
-  </si>
-  <si>
-    <t>У F-130 вказано мінімум 5 голосів, тоді як у BL-20 — 3. Це різні очікувані результати для тієї самої моделі. Пропоную прийняти поріг 3 голоси, узгодивши його із замовником. До погодження порогу тест-кейс матиме два результати.</t>
-  </si>
-  <si>
-    <t>Сеанс не може бути водночас безстроковим і завершуватися через 30 хвилин. Пропоную визначити завершення після 30 хвилин бездіяльності або натискання Logout. Це дозволить перевірити час очікування.</t>
-  </si>
-  <si>
-    <t>Правило зберігання паролів як хешів не має власного ID, тому на нього не можна посилатися з тестів. Пропоную додати ID S-15 без перенумерації інших вимог. Новий ID потрібний у матриці простежуваності.</t>
-  </si>
-  <si>
-    <t>F-120 повторює загальний рейтинг, який уже описано у F-70 та частково F-10. Дубль краще вилучити, залишивши номер F-120 вільним і зафіксувавши це в журналі змін. Один тест не повинен прив’язуватися до двох дублікатів.</t>
-  </si>
-  <si>
-    <t>F-100 посилається на BL-35, але такої вимоги в документі немає. Посилання потрібно замінити на наявну BL-30, щоб можна було простежити правило до тесту. Без цього зв’язок із BL-вимогою некоректний.</t>
-  </si>
-  <si>
-    <t>Перевірка даних через державні реєстри потребує інтеграцій, які для цього продукту не передбачені. Реально виконати локальну перевірку формату телефону, віку та довжини адреси. Після уточнення можна задати перевірювані вхідні дані.</t>
-  </si>
-  <si>
-    <t>Час 50 мс навіть у мережі 2G не залежить повністю від застосунку і не може гарантуватися. Пропоную міряти p95 ≤ 3 с у визначеному середовищі на каталозі до 1000 моделей. Умови мережі та вибірку необхідно записати в плані.</t>
-  </si>
-  <si>
-    <t>Поняття «працювати швидко» не можна перевірити без чисел. Потрібні вимірювані умови: p95 відкриття моделі ≤ 2,5 с, підтвердження голосу ≤ 2 с за 30 вимірів. Такі пороги дозволять фіксувати пройдено/не пройдено.</t>
-  </si>
-  <si>
-    <t>Твердження «інтуїтивно для будь-якого» неможливо підтвердити одним тестом. Пропоную критерій: щонайменше 4 з 5 новачків знаходять модель і можливість проголосувати за 3 хвилини. Отримаємо відтворюваний критерій юзабіліті.</t>
-  </si>
-  <si>
-    <t>Обіцянку заблокувати будь-яку спробу несанкціонованого доступу неможливо перевірити вичерпно. Слід описати конкретні заборони гостю й правило блокування після 5 невдалих входів за 15 хвилин. Такі перевірки реально внести до набору тест-кейсів.</t>
-  </si>
-  <si>
-    <t>Зараз не зрозуміло, як саме обираються Popular Make і Popular Model при однаковій кількості голосів. Пропоную визначати популярність за голосами, а при нічиїй сортувати назви за алфавітом. Для граничного випадку в тесті слід взяти дві моделі з однаковими голосами.</t>
-  </si>
-  <si>
-    <t>Фраза «достатньо складний пароль» допускає різні перевірки. Потрібно прямо записати умови: 8–64 символи, щонайменше одна латинська літера та одна цифра. Перевірити довжину 7, 8, 64 та 65 символів.</t>
-  </si>
-  <si>
-    <t>Не визначено, що вважати окремим словом зі стоп-списку. Варто перевіряти межі слова за літерами Unicode: «spam!» повинно збігатися зі словом spam, а «spammer» — ні. У юніт-тесті потрібні приклади з пунктуацією та вкладеним словом.</t>
-  </si>
-  <si>
-    <t>У F-40 описаний лише успішний вхід. Для помилки треба додати відмову в авторизації, збереження поточної сторінки та повідомлення «Invalid login or password». Окремий тест має перевіряти неправильні облікові дані.</t>
-  </si>
-  <si>
-    <t>Не описано, як виглядає рейтинг, коли немає жодної моделі. Пропоную показувати «No models found» і не відображати кнопки пагінації, щоб не було порожніх сторінок. Перевіряється відсутність пагінації за нульового результату.</t>
-  </si>
-  <si>
-    <t>Сортування моделей з однаковим rating не задане, тому порядок може змінюватися між запусками. Після рейтингу потрібно сортувати за повною назвою моделі без урахування регістру. Можна підготувати два записи з однаковим рейтингом.</t>
-  </si>
-  <si>
-    <t>У F-60 ранг залежить від кількості голосів, але F-130 використовує зважений рейтинг. Потрібно встановити єдине правило ранжування за рейтингом і узгодити його з BL-20. Слід створити модель з більшою кількістю, але нижчою зваженою оцінкою.</t>
-  </si>
-  <si>
-    <t>F-90 не дозволяє голосувати без коментаря, а BL-50 фактично пропускає порожнє значення. Модуль повинен відхиляти null, порожній рядок і рядок з одних пробілів. У тестах BL-50 окремо перевірити null, "" і пробіли.</t>
-  </si>
-  <si>
-    <t>У F-130 вказано мінімум 5 голосів, тоді як у BL-20 — 3. Це різні очікувані результати для тієї самої моделі. Пропоную прийняти поріг 3 голоси, узгодивши його із замовником. Граничними значеннями будуть 2, 3 і 4 голоси.</t>
-  </si>
-  <si>
-    <t>F-120 повторює загальний рейтинг, який уже описано у F-70 та частково F-10. Дубль краще вилучити, залишивши номер F-120 вільним і зафіксувавши це в журналі змін. Після вилучення перевірити посилання на F-70.</t>
-  </si>
-  <si>
-    <t>F-100 посилається на BL-35, але такої вимоги в документі немає. Посилання потрібно замінити на наявну BL-30, щоб можна було простежити правило до тесту. Юніт-тести треба прив’язати до чинної BL-30.</t>
-  </si>
-  <si>
-    <t>Перевірка даних через державні реєстри потребує інтеграцій, які для цього продукту не передбачені. Реально виконати локальну перевірку формату телефону, віку та довжини адреси. Зовнішні реєстри не можна вважати доступними для тестового стенда.</t>
-  </si>
-  <si>
-    <t>Гарантувати розпізнавання будь-яких помилок, транслітерації та наміру користувача неможливо. Доцільно обмежити пошук точним збігом префікса без урахування регістру. Описаний префіксний пошук можна перевірити на різному регістрі.</t>
-  </si>
-  <si>
-    <t>BL-80 не може працювати «без помилок» на абсолютно будь-яких аргументах. Треба визначити допустимі дані та очікувані винятки для некоректних значень. Для кожного некоректного аргументу потрібний визначений результат.</t>
-  </si>
-  <si>
-    <t>Правило активності Register описане нечітко, тому незрозуміло, коли її можна натиснути. Кнопка має ставати активною тільки після заповнення полів і успішної перевірки паролів за F-30. Після правки буде однакова умова перевірки на різних екранах.</t>
-  </si>
-  <si>
-    <t>Не визначено, що вважати окремим словом зі стоп-списку. Варто перевіряти межі слова за літерами Unicode: «spam!» повинно збігатися зі словом spam, а «spammer» — ні. Приклади збігів треба додати до контрольного списку.</t>
-  </si>
-  <si>
-    <t>Сортування моделей з однаковим rating не задане, тому порядок може змінюватися між запусками. Після рейтингу потрібно сортувати за повною назвою моделі без урахування регістру. Правило має бути однаковим у BL-70 та в тест-плані.</t>
-  </si>
-  <si>
-    <t>F-90 не дозволяє голосувати без коментаря, а BL-50 фактично пропускає порожнє значення. Модуль повинен відхиляти null, порожній рядок і рядок з одних пробілів. Після виправлення варто повторно звірити F-90.</t>
-  </si>
-  <si>
-    <t>GUI-60 дозволяє 10 рядків, а F-140 — 5, тому неможливо правильно перевірити пагінацію. Потрібно встановити однаковий розмір сторінки — 5 моделей. Так зникне розбіжність між GUI та функціональною вимогою.</t>
-  </si>
-  <si>
-    <t>Два різні правила мають ID GUI-40, через що посилання в тест-кейсах будуть неоднозначними. Перший ID треба зберегти, а другій вимозі надати GUI-45. Посилання на GUI-40 і GUI-45 після зміни слід перевірити.</t>
-  </si>
-  <si>
-    <t>Гарантувати розпізнавання будь-яких помилок, транслітерації та наміру користувача неможливо. Доцільно обмежити пошук точним збігом префікса без урахування регістру. Обмеження пошуку потрібно винести у відомі обмеження продукту.</t>
-  </si>
-  <si>
-    <t>BL-80 не може працювати «без помилок» на абсолютно будь-яких аргументах. Треба визначити допустимі дані та очікувані винятки для некоректних значень. Винятки варто описати однаково у вимогах і майбутніх тестах.</t>
-  </si>
-  <si>
-    <t>Слова «зручно» і «не викликає труднощів» не мають критерію успіху. Варто перевіряти на 5 користувачах: щонайменше 4 мають завершити редагування за 3 хвилини.</t>
-  </si>
-  <si>
-    <t>Правило активності Register описане нечітко, тому незрозуміло, коли її можна натиснути. Кнопка має ставати активною тільки після заповнення полів і успішної перевірки паролів за F-30. Зміна має бути узгоджена з F-30.</t>
-  </si>
-  <si>
-    <t>D-10 посилається на документ АР-СТД-07, якого немає серед матеріалів. Краще перелічити обов’язкові розділи довідки в самій SRS, щоб вимогу можна було перевірити. Потрібен визначений обсяг довідки для приймання роботи.</t>
-  </si>
-  <si>
-    <t>GUI-60 дозволяє 10 рядків, а F-140 — 5, тому неможливо правильно перевірити пагінацію. Потрібно встановити однаковий розмір сторінки — 5 моделей. Перед затвердженням закріпити єдине число 5.</t>
-  </si>
-  <si>
-    <t>Сеанс не може бути водночас безстроковим і завершуватися через 30 хвилин. Пропоную визначити завершення після 30 хвилин бездіяльності або натискання Logout. Це потрібно погодити як правило безпеки сеансу.</t>
-  </si>
-  <si>
-    <t>Два різні правила мають ID GUI-40, через що посилання в тест-кейсах будуть неоднозначними. Перший ID треба зберегти, а другій вимозі надати GUI-45. ID не можна перенумеровувати в інших вимогах.</t>
-  </si>
-  <si>
-    <t>Правило зберігання паролів як хешів не має власного ID, тому на нього не можна посилатися з тестів. Пропоную додати ID S-15 без перенумерації інших вимог. Зміна не повинна зачіпати наявні ID.</t>
-  </si>
-  <si>
-    <t>Час 50 мс навіть у мережі 2G не залежить повністю від застосунку і не може гарантуватися. Пропоную міряти p95 ≤ 3 с у визначеному середовищі на каталозі до 1000 моделей. Це реалістичніше з урахуванням роботи публічного demo.</t>
-  </si>
-  <si>
-    <t>Слова «зручно» і «не викликає труднощів» не мають критерію успіху. Варто перевіряти на 5 користувачах: щонайменше 4 мають завершити редагування за 3 хвилини. Критерій має застосовуватися до однакових завдань учасників.</t>
-  </si>
-  <si>
-    <t>Поняття «працювати швидко» не можна перевірити без чисел. Потрібні вимірювані умови: p95 відкриття моделі ≤ 2,5 с, підтвердження голосу ≤ 2 с за 30 вимірів. Перед виконанням замірів треба погодити умови стенда.</t>
-  </si>
-  <si>
-    <t>Твердження «інтуїтивно для будь-якого» неможливо підтвердити одним тестом. Пропоную критерій: щонайменше 4 з 5 новачків знаходять модель і можливість проголосувати за 3 хвилини. Учасники повинні отримати однаковий сценарій.</t>
-  </si>
-  <si>
-    <t>Обіцянку заблокувати будь-яку спробу несанкціонованого доступу неможливо перевірити вичерпно. Слід описати конкретні заборони гостю й правило блокування після 5 невдалих входів за 15 хвилин. Активні перевірки захищеності проводити лише на дозволеному стенді.</t>
+    <t>Хто знайшов</t>
+  </si>
+  <si>
+    <t>«Popular Make» визначається за найбільшою сумарною кількістю голосів за моделі марки, «Popular Model» — за найбільшою кількістю голосів за модель. За однакової кількості голосів обирається назва за алфавітом без урахування регістру.</t>
+  </si>
+  <si>
+    <t>Асташов Іван; Кінаш Єгор</t>
+  </si>
+  <si>
+    <t>Прийнято</t>
+  </si>
+  <si>
+    <t>Під час реєстрації система перевіряє, що всі поля заповнені, значення полів «Password» і «Confirm Password» збігаються, а пароль містить від 8 до 64 символів, щонайменше одну латинську літеру та одну цифру. У разі порушення система показує повідомлення про помилку під формою і не створює обліковий запис.</t>
+  </si>
+  <si>
+    <t>На сторінці реєстрації кнопка «Register» неактивна, поки хоча б одне обов’язкове поле порожнє, паролі не збігаються або пароль не відповідає F-30. Кнопка стає активною тільки після виконання всіх цих умов.</t>
+  </si>
+  <si>
+    <t>Рушай Євген; Дарина Поломарьова</t>
+  </si>
+  <si>
+    <t>Словом є послідовність літер Unicode; роздільники — будь-які інші символи. Збіг повного слова без урахування регістру: «spam!» заборонено, «spammer» — ні.</t>
+  </si>
+  <si>
+    <t>Кінаш Єгор; Рушай Євген</t>
+  </si>
+  <si>
+    <t>Якщо логін не існує або пароль неправильний, вхід не виконується, сторінка не змінюється і поряд із формою показується «Invalid login or password».</t>
+  </si>
+  <si>
+    <t>Якщо таблиця порожня, показується «No models found», пагінація не відображається.</t>
+  </si>
+  <si>
+    <t>ModelSearch.sortByRating(models): повертає новий список за спаданням числового рейтингу; для однакових рейтингів — за повною назвою (марка + модель) за алфавітом без урахування регістру. Оригінальний список не змінюється; null-колекція — IllegalArgumentException.</t>
+  </si>
+  <si>
+    <t>До пакета постачання входить довідка користувача українською мовою у форматі Markdown або PDF із розділами «Реєстрація та вхід», «Перегляд каталогу», «Голосування», «Профіль», «Типові помилки». Кожна дія має назву кнопки чи екрана, послідовність кроків і очікуваний результат; зовнішній стандарт оформлення для цієї версії не застосовується.</t>
+  </si>
+  <si>
+    <t>Асташов Іван; Дарина Поломарьова</t>
+  </si>
+  <si>
+    <t>Моделі з щонайменше 3 голосами отримують ранг за спаданням зваженого рейтингу BL-10; при однаковому рейтингу порядок визначається за повною назвою марки й моделі без урахування регістру (BL-20). Моделі з менш ніж 3 голосами відображаються після ранжованих із позначкою «—» у полі «Rank»; порядок серед них — за назвою.</t>
+  </si>
+  <si>
+    <t>Коментар обов’язковий: null, порожній рядок або рядок тільки з пробілів відхиляється з повідомленням «порожній коментар». Максимальна довжина — 200 символів Unicode; якщо перевищено — «коментар задовгий». Це правило однакове для вебформи та VoteValidator.validate.</t>
+  </si>
+  <si>
+    <t>Рейтинг моделі обчислюється як зважене середнє за BL-10. Ранги в межах марки і загального рейтингу визначаються за спаданням цього рейтингу з алфавітним правилом для рівних значень (BL-20). Для ранжування модель повинна мати щонайменше 3 зараховані голоси. Моделі з меншою кількістю голосів залишаються у каталозі, але не беруть участі в загальному ранжуванні.</t>
+  </si>
+  <si>
+    <t>Таблиці моделей розбиваються на сторінки по 5 рядків; елементи навігації ««», «»» і напис «page X of Y» розміщено безпосередньо під таблицею, вирівняно по центру.</t>
+  </si>
+  <si>
+    <t>Сеанс користувача завершується після натискання «Logout» або після 30 хвилин бездіяльності. Після завершення сеансу сторінка профілю й голосування недоступні до повторного входу. Активні дії користувача скидають таймер бездіяльності.</t>
+  </si>
+  <si>
+    <t>Друга вимога GUI-40 має ідентифікатор GUI-45: На сторінці профілю поля «Hobby» і «Language» реалізовано як випадні списки, поле «Age» приймає лише цілі невід'ємні числа; кнопка «Save» неактивна, доки жодне поле не змінено.</t>
+  </si>
+  <si>
+    <t>S-15: Паролі користувачів зберігаються лише у вигляді хешу; у відповідях сервера і в адресному рядку пароль не передається.</t>
+  </si>
+  <si>
+    <t>F-120 вилучено як дубль. Перелік моделей визначає F-70, перехід до нього — F-10. Ідентифікатор F-120 не використовується повторно.</t>
+  </si>
+  <si>
+    <t>Користувач може віддати лише один голос за кожну модель (правило BL-30): після зарахування голосу форма голосування на сторінці цієї моделі для цього користувача більше не відображається, а повторний голос відхиляється.</t>
+  </si>
+  <si>
+    <t>Вік — ціле число від 0 до 120, телефон — «+» та від 10 до 15 цифр, адреса — до 200 символів. Порушення формату блокує збереження і показує повідомлення біля поля. Дані не звіряються з державними реєстрами.</t>
+  </si>
+  <si>
+    <t>ModelSearch.search(query, models): пошук без урахування регістру за префіксом назви марки або моделі. Порожній, пробільний або null-запит повертає порожній список; null-колекція — IllegalArgumentException. Результати зберігають порядок вхідного списку. Виправлення описок, транслітерація та семантичний пошук не входять у версію 1.1.</t>
+  </si>
+  <si>
+    <t>Для null замість колекції методи викидають IllegalArgumentException. Некоректні оцінка та репутація в RatingAggregator.average обробляються за BL-10, а порушення правил голосу у VoteValidator.validate повертаються як повідомлення за BL-30, BL-40 і BL-50. ModelSearch.search для null-запиту повертає порожній список за BL-60.</t>
+  </si>
+  <si>
+    <t>На контрольованому тестовому середовищі (Chrome, 10 Мбіт/с, RTT 100 мс, каталог до 1 000 моделей) 95-й перцентиль повного завантаження сторінки Overall Rating не перевищує 3 с у 30 послідовних вимірюваннях. Час відповіді зовнішньої мережі з довільними параметрами не гарантується.</t>
+  </si>
+  <si>
+    <t>Форма профілю має видимі підписи для всіх полів, повідомлення про помилку розміщується безпосередньо біля відповідного поля, а збереження доступне з клавіатури. У перевірці на 5 нових користувачах щонайменше 4 мають змінити номер телефону і зберегти профіль за 3 хвилини без сторонньої допомоги.</t>
+  </si>
+  <si>
+    <t>На контрольованому тестовому стенді за одного активного користувача 95-й перцентиль часу відкриття сторінки моделі не перевищує 2,5 с, а часу підтвердження голосу — 2 с (по 30 вимірювань). Відлік — від дії користувача до відображення повного результату.</t>
+  </si>
+  <si>
+    <t>Під час перевірки на 5 нових користувачах не менше 4 учасників без інструктажу повинні знайти модель у каталозі, відкрити картку та визначити, як проголосувати, не довше ніж за 3 хвилини. Результат фіксує спостерігач; доступ до голосування можливий після входу.</t>
+  </si>
+  <si>
+    <t>Сторінка «Profile» та дія голосування потребують дійсного сеансу; без входу система відмовляє в доступі й не змінює дані. Після 5 невдалих спроб входу для одного логіна за 15 хвилин наступний вхід для нього блокується на 15 хвилин з повідомленням про тимчасове блокування. Перевіряють правильні і неправильні облікові дані та доступ за прямим URL.</t>
+  </si>
+  <si>
+    <t>Мінімум голосів — 3 чи 5?</t>
+  </si>
+  <si>
+    <t>Прийнято 3, оскільки саме так формулюється BL-20, який тестуватиметься JUnit.</t>
+  </si>
+  <si>
+    <t>Ранг залежить від голосів чи зваженої оцінки?</t>
+  </si>
+  <si>
+    <t>Для рангу — зважений рейтинг за BL-10; Popular Model за кількістю голосів (F-10).</t>
+  </si>
+  <si>
+    <t>Яка точна складність пароля?</t>
+  </si>
+  <si>
+    <t>8–64 символи, щонайменше одна латинська літера й одна цифра; правило зафіксовано у F-30.</t>
+  </si>
+  <si>
+    <t>Ліміти невдалого входу і тривалість сеансу?</t>
+  </si>
+  <si>
+    <t>5 спроб за 15 хв / блок 15 хв, завершення після 30 хв бездіяльності.</t>
+  </si>
+  <si>
+    <t>Чи прийнятні контрольовані пороги p95 та середовище?</t>
+  </si>
+  <si>
+    <t>P-10: p95 ≤3 с; P-20: відкриття моделі ≤2,5 с, підтвердження голосу ≤2 с. Контрольоване середовище, по 30 вимірювань.</t>
+  </si>
+  <si>
+    <t>Чи можна вилучити дубль вимоги?</t>
+  </si>
+  <si>
+    <t>Так: весь зміст F-120 покритий F-70 і F-10, ID не використовується повторно.</t>
+  </si>
+  <si>
+    <t>Коментар обов’язковий на всіх рівнях?</t>
+  </si>
+  <si>
+    <t>Так, інакше через модуль можна прийняти голос без коментаря.</t>
+  </si>
+  <si>
+    <t>Запис / RD — Асташов Іван</t>
+  </si>
+  <si>
+    <t>Підстава у SRS 1.0</t>
+  </si>
+  <si>
+    <t>Результат перевірки</t>
+  </si>
+  <si>
+    <t>Висновок</t>
+  </si>
+  <si>
+    <t>Дата запису</t>
+  </si>
+  <si>
+    <t>ТА-01 / RD-01</t>
+  </si>
+  <si>
+    <t>Стор. 3, F-10: «Popular Make»; «Popular Model» — спосіб визначення популярності не заданий.</t>
+  </si>
+  <si>
+    <t>Затверджено</t>
+  </si>
+  <si>
+    <t>F-10 описує вміст блоків, але не спосіб вибору популярної марки й моделі. У редакції 1.1 популярність визначається кількістю голосів, а рівні значення — алфавітним порядком назв.</t>
+  </si>
+  <si>
+    <t>ТА-02 / RD-02</t>
+  </si>
+  <si>
+    <t>Стор. 3, F-30: «пароль є достатньо складним»</t>
+  </si>
+  <si>
+    <t>Вислів «достатньо складним» не задає обмежень довжини або складу пароля. F-30 тепер прямо визначає 8–64 символи, латинську літеру та цифру; інші поля й поведінка помилки збережені.</t>
+  </si>
+  <si>
+    <t>ТА-03 / RD-05</t>
+  </si>
+  <si>
+    <t>Стор. 3, F-40: Описано лише успішний вхід; результат для неправильних даних відсутній.</t>
+  </si>
+  <si>
+    <t>F-40 містить тільки успішний вхід; GUI-30 описує розміщення помилки, але не результат авторизації. Додано явну відмову, збереження поточної сторінки й текст «Invalid login or password».</t>
+  </si>
+  <si>
+    <t>ТА-04 / RD-06</t>
+  </si>
+  <si>
+    <t>Стор. 4, F-140: Визначені сторінки по 5 рядків; стан таблиці з 0 моделей відсутній.</t>
+  </si>
+  <si>
+    <t>F-140 задає навігацію першою й останньою сторінкою, але не визначає стан порожнього каталогу. Для нуля моделей тепер встановлено текст «No models found» і відсутність пагінації.</t>
+  </si>
+  <si>
+    <t>ТА-05 / RD-08</t>
+  </si>
+  <si>
+    <t>Стор. 6, D-10: «відповідно до стандарту оформлення документації «АР-СТД-07»»</t>
+  </si>
+  <si>
+    <t>D-10 вимагає відповідності АР-СТД-07, однак текст стандарту не входить до вихідних матеріалів. Його замінено самодостатнім переліком п’яти розділів довідки, формату та змісту опису кожної дії.</t>
+  </si>
+  <si>
+    <t>ТА-06 / RD-09</t>
+  </si>
+  <si>
+    <t>Стор. 3, F-60: F-60: «ранг 1 має модель із найбільшою кількістю голосів»; F-130 / BL-20: спадання рейтингу.</t>
+  </si>
+  <si>
+    <t>F-60 і термін «Ранг» визначали перше місце кількістю голосів, а F-130 та BL-20 — зваженим рейтингом. Встановлено рейтинг за BL-10 і правило рівності BL-20; F-70 та словник приведено до цього визначення.</t>
+  </si>
+  <si>
+    <t>ТА-07 / RD-11</t>
+  </si>
+  <si>
+    <t>Стор. 4, F-130: F-130: «щонайменше 5 голосів»; BL-20: «лише з ≥3 голосами».</t>
+  </si>
+  <si>
+    <t>У F-130 поріг дорівнював 5 голосам, у BL-20 — 3. Для редакції 1.1 прийнято 3 голоси. Моделі з меншою кількістю лишаються в каталозі без рангу; F-60 і F-70 мають таку саму умову.</t>
+  </si>
+  <si>
+    <t>ТА-08 / RD-13</t>
+  </si>
+  <si>
+    <t>Стор. 6, S-20: «зберігається безстроково»; «після 30 хвилин неактивності сеанс автоматично завершується».</t>
+  </si>
+  <si>
+    <t>У S-20 одночасно вказані безстроковість і завершення після 30 хвилин. Безстроковість вилучено: завершення настає після Logout або 30 хвилин бездіяльності; визначення сеансу оновлено.</t>
+  </si>
+  <si>
+    <t>ТА-09 / RD-15</t>
+  </si>
+  <si>
+    <t>Стор. 6, розд. 6, без ID: Паролі користувачів зберігаються лише у вигляді хешу; у відповідях сервера і в адресному рядку пароль не передається.</t>
+  </si>
+  <si>
+    <t>Рядок про хешування та непередавання пароля у відповідях і адресному рядку не мав ID. Йому присвоєно S-15. Текст вимоги та пріоритет High збережені дослівно.</t>
+  </si>
+  <si>
+    <t>ТА-10 / RD-16</t>
+  </si>
+  <si>
+    <t>Стор. 4, F-120: F-120 повторює перехід через Overall Rating із F-10 і таблицю моделей із F-70.</t>
+  </si>
+  <si>
+    <t>F-120 повторює перехід із F-10 та таблицю загального рейтингу з F-70. Дубль вилучено, а номер F-120 залишено невикористаним; у журналі наведено повний вилучений текст.</t>
+  </si>
+  <si>
+    <t>ТА-11 / RD-17</t>
+  </si>
+  <si>
+    <t>Стор. 3, F-100: «Користувач може віддати лише один голос за кожну модель (правило BL-35)»</t>
+  </si>
+  <si>
+    <t>У F-100 була пряма вказівка на відсутню BL-35. Посилання замінено на BL-30; решту тексту F-100 збережено, тому правило одного голосу не змінило змісту.</t>
+  </si>
+  <si>
+    <t>ТА-12 / RD-18</t>
+  </si>
+  <si>
+    <t>Стор. 4, F-110: «перевіряє достовірність указаних адреси, телефону та віку за державними реєстрами»</t>
+  </si>
+  <si>
+    <t>F-110 вимагала автоматичних перевірок у державних реєстрах без заданих інтеграцій. Прийняті локальні правила: вік 0–120, телефон із «+» і 10–15 цифрами, адреса до 200 символів та помилка біля поля.</t>
+  </si>
+  <si>
+    <t>ТА-13 / RD-21</t>
+  </si>
+  <si>
+    <t>Стор. 5, P-10: «не довше ніж за 50 мс за будь-якого з’єднання, включно з мобільним 2G»</t>
+  </si>
+  <si>
+    <t>P-10 поєднувала 50 мс, довільну мережу та довільний каталог. Прийнято 30 вимірювань, p95 ≤3 с, Chrome, 10 Мбіт/с, RTT 100 мс і до 1000 моделей. Умови додані до розділів 2.2–2.3.</t>
+  </si>
+  <si>
+    <t>ТА-14 / RD-23</t>
+  </si>
+  <si>
+    <t>Стор. 6, P-20: Система має працювати швидко і без затримок під час голосування та перегляду сторінок моделей.</t>
+  </si>
+  <si>
+    <t>P-20 містила тільки слово «швидко». Визначено відлік від дії до повного результату, одного активного користувача і 30 замірів для кожної операції: p95 ≤2,5 с для моделі та ≤2 с для голосу.</t>
+  </si>
+  <si>
+    <t>ТА-15 / RD-24</t>
+  </si>
+  <si>
+    <t>Стор. 6, U-10: Інтерфейс має бути інтуїтивно зрозумілим для будь-якого користувача.</t>
+  </si>
+  <si>
+    <t>U-10 обіцяла зрозумілість будь-якому користувачеві без критерію. Встановлено сценарій пошуку моделі й способу голосування, 5 новачків, поріг 4 успішних учасників і ліміт 3 хвилини.</t>
+  </si>
+  <si>
+    <t>ТА-16 / RD-25</t>
+  </si>
+  <si>
+    <t>Стор. 6, S-10: Система має унеможливити будь-які спроби несанкціонованого доступу до облікових записів, включно з підбором пароля.</t>
+  </si>
+  <si>
+    <t>S-10 містила неперевірювану абсолютну гарантію. Її замінено відмовою гостю в доступі до Profile і голосування та правилом 5 помилок за 15 хвилин із блокуванням логіна на 15 хвилин.</t>
+  </si>
+  <si>
+    <t>Запис / RD — Кінаш Єгор</t>
+  </si>
+  <si>
+    <t>ІТ-01 / RD-01</t>
+  </si>
+  <si>
+    <t>Для двох моделей з однаковою кількістю голосів SRS 1.0 не дає єдиного очікуваного переможця. Після правки однакова фікстура завжди обирає першу назву за алфавітом без урахування регістру.</t>
+  </si>
+  <si>
+    <t>ІТ-02 / RD-02</t>
+  </si>
+  <si>
+    <t>Границі для перевірки F-30 — 7, 8, 64 і 65 символів. Окремі негативні набори: без латинської літери та без цифри. Після правки для кожного набору визначено прийняття або відмову.</t>
+  </si>
+  <si>
+    <t>ІТ-03 / RD-04</t>
+  </si>
+  <si>
+    <t>Стор. 5, BL-80: «окреме слово зі стоп-списку»</t>
+  </si>
+  <si>
+    <t>Для стоп-слова spam контрольні приклади мають різні результати: «SPAM!» відхиляється, «spammer» дозволено. Редакція BL-80 фіксує ці результати через збіг цілого слова з літер Unicode без урахування регістру.</t>
+  </si>
+  <si>
+    <t>ІТ-04 / RD-05</t>
+  </si>
+  <si>
+    <t>Негативні набори для F-40 — неіснуючий логін і правильний логін з неправильним паролем. Обидва залишають користувача гостем на тій самій сторінці з однаковим повідомленням помилки.</t>
+  </si>
+  <si>
+    <t>ІТ-05 / RD-06</t>
+  </si>
+  <si>
+    <t>Фікстура з 0 моделей не мала визначеного очікуваного UI. У редакції 1.1 перевіряються повідомлення «No models found» і відсутність обох кнопок переходу; порожня сторінка не рахується як сторінка моделей.</t>
+  </si>
+  <si>
+    <t>ІТ-06 / RD-07</t>
+  </si>
+  <si>
+    <t>Стор. 5, BL-70: «за рейтингом за спаданням»; вторинний ключ для рівних рейтингів відсутній.</t>
+  </si>
+  <si>
+    <t>Для BL-70 два CarModel з однаковим rating могли повертатися в довільному порядку. Вторинний ключ тепер складається з марки й назви моделі без урахування регістру; вихідний список залишається незмінним.</t>
+  </si>
+  <si>
+    <t>ІТ-07 / RD-09</t>
+  </si>
+  <si>
+    <t>Контрольний приклад: модель із більшою кількістю голосів, але нижчим рейтингом не повинна отримати ранг 1. F-60 тепер узгоджується з BL-10/BL-20; кількість голосів залишається критерієм популярності F-10.</t>
+  </si>
+  <si>
+    <t>ІТ-08 / RD-10</t>
+  </si>
+  <si>
+    <t>Стор. 5, BL-50: BL-50: «порожній коментар (або null ) дозволено»; F-90: коментар обов’язковий.</t>
+  </si>
+  <si>
+    <t>Фікстури null, порожнього рядка та пробілів для коментаря тепер повертають «порожній коментар». Довжина 200 дозволена, 201 повертає «коментар задовгий». Це узгоджує результати валідатора з формою F-90.</t>
+  </si>
+  <si>
+    <t>ІТ-09 / RD-11</t>
+  </si>
+  <si>
+    <t>На 2 голосах модель не ранжується, на 3 і 4 — ранжується. Такі границі тепер однакові для F-130 та RatingAggregator.topN, тому перевірки UI і модуля більше не мають різних порогів.</t>
+  </si>
+  <si>
+    <t>ІТ-10 / RD-16</t>
+  </si>
+  <si>
+    <t>Після вилучення F-120 перевірки відкриття списку посилаються на F-10, а його вмісту — на F-70. Покриття сценарію збережене; прив’язка одного правила до двох дублікатів більше не потрібна.</t>
+  </si>
+  <si>
+    <t>ІТ-11 / RD-17</t>
+  </si>
+  <si>
+    <t>Для двох голосів з однаковою парою userId/modelId F-100 тепер веде до реалізованого контракту BL-30: другий голос відхиляється з повідомленням «повторний голос».</t>
+  </si>
+  <si>
+    <t>ІТ-12 / RD-18</t>
+  </si>
+  <si>
+    <t>Для профілю тепер можна підготувати відтворювані набори: вік −1/0/120/121, телефон із 9/10/15/16 цифрами та адресу 200/201 символ. Доступ до державних реєстрів для цих перевірок не потрібний.</t>
+  </si>
+  <si>
+    <t>ІТ-13 / RD-19</t>
+  </si>
+  <si>
+    <t>Стор. 5, BL-60: «розпізнавати запити з друкарськими помилками, транслітерацією та будь-якою мовою світу»</t>
+  </si>
+  <si>
+    <t>BL-60 тепер має визначений контракт: префікс марки або моделі без регістру, збереження вхідного порядку, порожній результат для порожнього, пробільного або null-запиту. Семантичне розпізнавання вилучено.</t>
+  </si>
+  <si>
+    <t>ІТ-14 / RD-20</t>
+  </si>
+  <si>
+    <t>Стор. 5, BL-80: «Модуль загалом має працювати без помилок за будь-яких вхідних даних».</t>
+  </si>
+  <si>
+    <t>Абсолютну обіцянку відсутності помилок замінено контрактами: null-колекція дає IllegalArgumentException, помилки голосу — повідомлення валідатора, null-запит пошуку — порожній список. Виняток і бізнес-відмову розмежовано.</t>
+  </si>
+  <si>
+    <t>Запис / RD — Рушай Євген</t>
+  </si>
+  <si>
+    <t>СМ-01 / RD-03</t>
+  </si>
+  <si>
+    <t>Стор. 4, GUI-20: «доки форму не заповнено належним чином»</t>
+  </si>
+  <si>
+    <t>Фраза GUI-20 «належним чином» не визначає умови активності Register. У виправленні перелічено заповнення обов’язкових полів, збіг паролів і виконання F-30; неповний набір умов залишає кнопку неактивною.</t>
+  </si>
+  <si>
+    <t>СМ-02 / RD-04</t>
+  </si>
+  <si>
+    <t>У BL-80 не було визначення меж слова. Тепер літери Unicode утворюють слово, а решта символів розділяє слова. Приклади з пунктуацією та частиною довшого слова включені без зміни переліку стоп-слів.</t>
+  </si>
+  <si>
+    <t>СМ-03 / RD-07</t>
+  </si>
+  <si>
+    <t>Сортування BL-70 у джерелі описувало тільки спадання рейтингу. Правило рівних значень доповнено повною назвою за алфавітом, що узгоджує його з уже наявною BL-20.</t>
+  </si>
+  <si>
+    <t>СМ-04 / RD-10</t>
+  </si>
+  <si>
+    <t>BL-50 прямо дозволяла порожній коментар і null, на відміну від F-90. Виправлена вимога робить коментар обов’язковим для вебформи й модуля та зберігає межу довжини 200 символів.</t>
+  </si>
+  <si>
+    <t>СМ-05 / RD-12</t>
+  </si>
+  <si>
+    <t>Стор. 4, GUI-60: GUI-60: «по 10 рядків»; F-140: «по 5 рядків».</t>
+  </si>
+  <si>
+    <t>GUI-60 визначала 10 рядків, хоча F-140 вимагала 5. У GUI-60 змінено лише розмір сторінки на 5; положення навігації та написи збережені.</t>
+  </si>
+  <si>
+    <t>СМ-06 / RD-14</t>
+  </si>
+  <si>
+    <t>Стор. 4, GUI-40 (2-й): Два GUI-40: правило обов’язкових полів реєстрації та правило елементів профілю.</t>
+  </si>
+  <si>
+    <t>Перший GUI-40 описує обов’язкові поля реєстрації, другий — елементи профілю. Профіль отримав GUI-45 із дослівно збереженим текстом; GUI-40 та інші номери не змінені.</t>
+  </si>
+  <si>
+    <t>СМ-07 / RD-19</t>
+  </si>
+  <si>
+    <t>У BL-60 обіцялося розпізнавання будь-яких описок, мов і наміру користувача. Обсяг звужено до перевірюваного префіксного пошуку; вимогу гарантувати довільний намір у редакції 1.1 відсутньо.</t>
+  </si>
+  <si>
+    <t>СМ-08 / RD-20</t>
+  </si>
+  <si>
+    <t>BL-80 більше не суперечить BL-10 та вступу розділу 5, де вже передбачено IllegalArgumentException. Некоректні дані обробляються за визначеними правилами відповідного методу.</t>
+  </si>
+  <si>
+    <t>СМ-09 / RD-22</t>
+  </si>
+  <si>
+    <t>Стор. 4, GUI-70: Форма профілю має бути зручною для заповнення і не викликати труднощів у користувача.</t>
+  </si>
+  <si>
+    <t>GUI-70 не мала спостережуваного критерію зручності. Тепер визначені видимі підписи, помилки біля полів, збереження з клавіатури та результат щонайменше 4 із 5 учасників за 3 хвилини.</t>
+  </si>
+  <si>
+    <t>Запис / RD — Дарина Поломарьова</t>
+  </si>
+  <si>
+    <t>КТ-01 / RD-03</t>
+  </si>
+  <si>
+    <t>Умова приймання GUI-20 тепер збігається з F-30: Register доступна лише після всіх перевірок форми. Для порожнього поля, різних паролів і порушення складності очікується неактивна кнопка.</t>
+  </si>
+  <si>
+    <t>КТ-02 / RD-08</t>
+  </si>
+  <si>
+    <t>Для приймання D-10 тепер достатньо перевірити наявність п’яти названих розділів, назв екранів і кнопок, кроків та результату. Посилання на ненаданий зовнішній стандарт вилучене.</t>
+  </si>
+  <si>
+    <t>КТ-03 / RD-12</t>
+  </si>
+  <si>
+    <t>Прийнята місткість сторінки — 5 моделей. Вибірка з 5 моделей має одну сторінку, з 6 — дві; вимоги GUI-60 і F-140 тепер дають однакові очікувані результати.</t>
+  </si>
+  <si>
+    <t>КТ-04 / RD-13</t>
+  </si>
+  <si>
+    <t>Для S-20 прийнято таймер бездіяльності на 30 хвилин із перезапуском після активних дій. Після тайм-ауту профіль і голосування потребують нового входу; Logout завершує сеанс одразу.</t>
+  </si>
+  <si>
+    <t>КТ-05 / RD-14</t>
+  </si>
+  <si>
+    <t>Для кожного правила форми тепер існує окремий ID. Посилання на обов’язковість реєстрації веде до GUI-40, на випадні списки й Save у профілі — до GUI-45; дубль усунуто без перенумерації.</t>
+  </si>
+  <si>
+    <t>КТ-06 / RD-15</t>
+  </si>
+  <si>
+    <t>Правило зберігання й передавання пароля тепер простежується за S-15 із реєстру до специфікації та майбутніх кейсів. Ідентифікатори S-10 і S-20 залишилися без змін.</t>
+  </si>
+  <si>
+    <t>КТ-07 / RD-21</t>
+  </si>
+  <si>
+    <t>Критерій приймання P-10 застосовується тільки до контрольованого середовища з названими параметрами. Вимір довільного публічного з’єднання не підмінює цей критерій; навантаження на спільний demo не планується.</t>
+  </si>
+  <si>
+    <t>КТ-08 / RD-22</t>
+  </si>
+  <si>
+    <t>Однакове завдання для приймання GUI-70 — змінити телефон і зберегти профіль без допомоги. Критерій проходження: не менше 4 із 5 нових користувачів вкладаються в 3 хвилини.</t>
+  </si>
+  <si>
+    <t>КТ-09 / RD-23</t>
+  </si>
+  <si>
+    <t>Показники відкриття моделі й підтвердження голосу тепер вимірюються окремо на контрольованому стенді. Кожна операція має власний поріг і вибірку із 30 вимірювань; результати між операціями не змішуються.</t>
+  </si>
+  <si>
+    <t>КТ-10 / RD-24</t>
+  </si>
+  <si>
+    <t>Для приймання U-10 спостерігач фіксує результат однакового завдання без інструктажу. Успіх — щонайменше 4 з 5 учасників знаходять модель, відкривають картку та визначають спосіб голосування за 3 хвилини.</t>
+  </si>
+  <si>
+    <t>КТ-11 / RD-25</t>
+  </si>
+  <si>
+    <t>Прийняті критерії S-10 визначають конкретні стани: гість не змінює дані, прямий URL профілю потребує сеансу, після порогу помилок вхід тимчасово блокується. Активні перевірки виконуються на окремому стенді.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -864,47 +1107,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
-    <cellStyle name="Normal" xfId="1"/>
-    <cellStyle name="Normal 2" xfId="3"/>
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 2" xfId="2"/>
-    <cellStyle name="Обычный 3" xfId="4"/>
-    <cellStyle name="Обычный 4" xfId="5"/>
-    <cellStyle name="Обычный 5" xfId="6"/>
-    <cellStyle name="Обычный 6" xfId="7"/>
+    <cellStyle name="Обычный 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Обычный 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Обычный 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Обычный 5" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Обычный 6" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -920,9 +1154,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -972,7 +1206,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1113,7 +1347,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -1129,32 +1363,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="78" customHeight="1">
@@ -1162,28 +1396,28 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="78" customHeight="1">
@@ -1191,28 +1425,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="78" customHeight="1">
@@ -1220,28 +1454,28 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>26</v>
+        <v>156</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="78" customHeight="1">
@@ -1249,28 +1483,28 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>31</v>
+        <v>157</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>158</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="78" customHeight="1">
@@ -1278,28 +1512,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>38</v>
+        <v>159</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="78" customHeight="1">
@@ -1307,28 +1541,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="78" customHeight="1">
@@ -1336,28 +1570,28 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>46</v>
+        <v>161</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="78" customHeight="1">
@@ -1365,28 +1599,28 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>51</v>
+        <v>162</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>32</v>
+        <v>163</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="78" customHeight="1">
@@ -1394,28 +1628,28 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>164</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="78" customHeight="1">
@@ -1423,28 +1657,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>61</v>
+        <v>165</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>21</v>
+        <v>158</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="78" customHeight="1">
@@ -1452,28 +1686,28 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>65</v>
+        <v>166</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>26</v>
+        <v>152</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="78" customHeight="1">
@@ -1481,28 +1715,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="F13" s="2" t="s">
-        <v>69</v>
+        <v>167</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="78" customHeight="1">
@@ -1510,28 +1744,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>74</v>
+        <v>168</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="78" customHeight="1">
@@ -1539,28 +1773,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="78" customHeight="1">
@@ -1568,28 +1802,28 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>84</v>
+        <v>170</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>26</v>
+        <v>163</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="78" customHeight="1">
@@ -1597,28 +1831,28 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>89</v>
+        <v>171</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="78" customHeight="1">
@@ -1626,28 +1860,28 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>93</v>
+        <v>172</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="78" customHeight="1">
@@ -1655,28 +1889,28 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>98</v>
+        <v>173</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>21</v>
+        <v>152</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="78" customHeight="1">
@@ -1684,28 +1918,28 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>102</v>
+        <v>174</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="78" customHeight="1">
@@ -1713,28 +1947,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>105</v>
+        <v>175</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>32</v>
+        <v>158</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="78" customHeight="1">
@@ -1742,28 +1976,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>109</v>
+        <v>176</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="78" customHeight="1">
@@ -1771,28 +2005,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>115</v>
+        <v>177</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="78" customHeight="1">
@@ -1800,28 +2034,28 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>119</v>
+        <v>178</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>26</v>
+        <v>163</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="78" customHeight="1">
@@ -1829,72 +2063,67 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>32</v>
+        <v>163</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="78" customHeight="1">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="85.5" customHeight="1">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>127</v>
+        <v>180</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="H2:H26">
-      <formula1>"прийнято,відхилено після обговорення,потребує рішення"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -1905,101 +2134,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
-      <c r="A1" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>132</v>
+      <c r="A1" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>137</v>
+        <v>110</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>142</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2008,7 +2237,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -2021,163 +2250,163 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>7</v>
+      <c r="B1" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>150</v>
+        <v>123</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>157</v>
+        <v>183</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>162</v>
+        <v>129</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>167</v>
+        <v>132</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>170</v>
+        <v>134</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>174</v>
+        <v>136</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>176</v>
+        <v>137</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>178</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="68.099999999999994" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>179</v>
+        <v>138</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>180</v>
+        <v>139</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>182</v>
+        <v>140</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>178</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2186,7 +2415,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -2197,22 +2426,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>186</v>
+      <c r="B1" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A2)</f>
@@ -2228,7 +2457,7 @@
     </row>
     <row r="3" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A3)</f>
@@ -2244,7 +2473,7 @@
     </row>
     <row r="4" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="B4" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A4)</f>
@@ -2260,7 +2489,7 @@
     </row>
     <row r="5" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A5)</f>
@@ -2276,7 +2505,7 @@
     </row>
     <row r="6" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="B6" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A6)</f>
@@ -2292,7 +2521,7 @@
     </row>
     <row r="7" spans="1:4" ht="33.950000000000003" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="B7" s="2">
         <f>COUNTIF(Реєстр!$C$2:$C$26,A7)</f>
@@ -2308,7 +2537,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
-        <v>187</v>
+        <v>144</v>
       </c>
       <c r="B9" s="4">
         <f>COUNT(Реєстр!A2:A26)</f>
@@ -2317,7 +2546,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="B10" s="4">
         <v>16</v>
@@ -2325,7 +2554,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>189</v>
+        <v>146</v>
       </c>
       <c r="B11" s="4">
         <v>40</v>
@@ -2333,7 +2562,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="B12" s="4">
         <v>7</v>
@@ -2341,7 +2570,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>191</v>
+        <v>148</v>
       </c>
       <c r="B13" s="4">
         <v>20</v>
@@ -2349,7 +2578,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>192</v>
+        <v>149</v>
       </c>
       <c r="B14" s="4">
         <v>24</v>
@@ -2361,7 +2590,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -2376,393 +2605,393 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="69.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>200</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>201</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="8">
-        <v>46308</v>
+        <v>203</v>
+      </c>
+      <c r="G2" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="69.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>204</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>19</v>
+        <v>205</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="G3" s="8">
-        <v>46308</v>
+        <v>206</v>
+      </c>
+      <c r="G3" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="69.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>39</v>
+        <v>207</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>37</v>
+        <v>208</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="G4" s="8">
-        <v>46308</v>
+        <v>209</v>
+      </c>
+      <c r="G4" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="69.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>210</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>41</v>
+        <v>211</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="G5" s="8">
-        <v>46308</v>
+        <v>212</v>
+      </c>
+      <c r="G5" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="69.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>52</v>
+        <v>213</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>50</v>
+        <v>214</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="G6" s="8">
-        <v>46308</v>
+        <v>215</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="69.95" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>216</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>217</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="G7" s="8">
-        <v>46308</v>
+        <v>218</v>
+      </c>
+      <c r="G7" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>66</v>
+        <v>219</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>64</v>
+        <v>220</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="G8" s="8">
-        <v>46308</v>
+        <v>221</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69.95" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>75</v>
+        <v>222</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>73</v>
+        <v>223</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="G9" s="8">
-        <v>46308</v>
+        <v>224</v>
+      </c>
+      <c r="G9" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>85</v>
+        <v>225</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>83</v>
+        <v>226</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="G10" s="8">
-        <v>46308</v>
+        <v>227</v>
+      </c>
+      <c r="G10" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="69.95" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>90</v>
+        <v>228</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>88</v>
+        <v>229</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="G11" s="8">
-        <v>46308</v>
+        <v>230</v>
+      </c>
+      <c r="G11" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="69.95" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>94</v>
+        <v>231</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>92</v>
+        <v>232</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="G12" s="8">
-        <v>46308</v>
+        <v>233</v>
+      </c>
+      <c r="G12" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="69.95" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>99</v>
+        <v>234</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>97</v>
+        <v>235</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G13" s="8">
-        <v>46308</v>
+        <v>236</v>
+      </c>
+      <c r="G13" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="69.95" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>110</v>
+        <v>237</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>108</v>
+        <v>238</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="G14" s="8">
-        <v>46308</v>
+        <v>239</v>
+      </c>
+      <c r="G14" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="69.95" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>118</v>
+        <v>241</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="G15" s="8">
-        <v>46308</v>
+        <v>242</v>
+      </c>
+      <c r="G15" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="69.95" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>124</v>
+        <v>243</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>122</v>
+        <v>244</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="G16" s="8">
-        <v>46308</v>
+        <v>245</v>
+      </c>
+      <c r="G16" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="69.95" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>128</v>
+        <v>246</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>126</v>
+        <v>247</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="G17" s="8">
-        <v>46308</v>
+        <v>248</v>
+      </c>
+      <c r="G17" s="7">
+        <v>46309</v>
       </c>
     </row>
   </sheetData>
@@ -2771,7 +3000,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -2786,347 +3015,347 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>199</v>
+        <v>249</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="69.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>250</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>201</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="G2" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="G2" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="69.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>252</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>19</v>
+        <v>205</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="G3" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="G3" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="69.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>254</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>30</v>
+        <v>255</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="G4" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="G4" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="69.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>257</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>37</v>
+        <v>208</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G5" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="G5" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="69.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>259</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>41</v>
+        <v>211</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="G6" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="69.95" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>261</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>45</v>
+        <v>262</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="G7" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="G7" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>58</v>
+        <v>264</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>56</v>
+        <v>217</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="G8" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69.95" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>266</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>60</v>
+        <v>267</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="G9" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="G9" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>66</v>
+        <v>269</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>64</v>
+        <v>220</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="G10" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G10" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="69.95" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>90</v>
+        <v>271</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>88</v>
+        <v>229</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="G11" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="G11" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="69.95" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>94</v>
+        <v>273</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>92</v>
+        <v>232</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="G12" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="G12" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="69.95" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>99</v>
+        <v>275</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>97</v>
+        <v>235</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="G13" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="G13" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="69.95" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>103</v>
+        <v>277</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>101</v>
+        <v>278</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="G14" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="G14" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="69.95" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>106</v>
+        <v>280</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>104</v>
+        <v>281</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="G15" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="G15" s="7">
+        <v>46309</v>
       </c>
     </row>
   </sheetData>
@@ -3135,7 +3364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -3150,232 +3379,232 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>200</v>
+        <v>283</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="69.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>284</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>285</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="G2" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="G2" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="69.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>287</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>30</v>
+        <v>255</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="G3" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="G3" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="69.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>289</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>45</v>
+        <v>262</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="G4" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="G4" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="69.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>62</v>
+        <v>291</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>60</v>
+        <v>267</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="G5" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="G5" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="69.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>293</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>68</v>
+        <v>294</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="G6" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="69.95" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>81</v>
+        <v>296</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>79</v>
+        <v>297</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="G7" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G7" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>103</v>
+        <v>299</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>101</v>
+        <v>278</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="G8" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69.95" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>106</v>
+        <v>301</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>104</v>
+        <v>281</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="G9" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>116</v>
+        <v>303</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>114</v>
+        <v>304</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="G10" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="G10" s="7">
+        <v>46309</v>
       </c>
     </row>
   </sheetData>
@@ -3384,7 +3613,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -3399,278 +3628,278 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>201</v>
+        <v>306</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="69.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>307</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>285</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="G2" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G2" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="69.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>52</v>
+        <v>309</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>50</v>
+        <v>214</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="G3" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="G3" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="69.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>70</v>
+        <v>311</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>68</v>
+        <v>294</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="G4" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="G4" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="69.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>75</v>
+        <v>313</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>73</v>
+        <v>223</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>244</v>
-      </c>
-      <c r="G5" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="G5" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="69.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>315</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>79</v>
+        <v>297</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="G6" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="69.95" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>85</v>
+        <v>317</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>83</v>
+        <v>226</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="G7" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="G7" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>110</v>
+        <v>319</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>108</v>
+        <v>238</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>247</v>
-      </c>
-      <c r="G8" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69.95" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>116</v>
+        <v>321</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>114</v>
+        <v>304</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="G9" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="G9" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>120</v>
+        <v>323</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>118</v>
+        <v>241</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="G10" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="G10" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="69.95" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>124</v>
+        <v>325</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>122</v>
+        <v>244</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="G11" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="G11" s="7">
+        <v>46309</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="69.95" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>128</v>
+        <v>327</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>126</v>
+        <v>247</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="8">
-        <v>46308</v>
+        <v>202</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="G12" s="7">
+        <v>46309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>